<commit_message>
str format for set number in find files
</commit_message>
<xml_diff>
--- a/тесты/исх для теста/выгрузки/Выгрузка комплекта №1 К-9.xlsx
+++ b/тесты/исх для теста/выгрузки/Выгрузка комплекта №1 К-9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\Project_OOD\тесты\исх для теста\выгрузки\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78832AC-122B-41E1-BB79-04007C0600BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87EA235-8600-452F-B3BF-6C45BE454930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4020" yWindow="2424" windowWidth="19020" windowHeight="9816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Выгрузка комплекта" sheetId="1" r:id="rId1"/>
@@ -28,58 +28,58 @@
     <t>СН комплекта</t>
   </si>
   <si>
+    <t>0012765490</t>
+  </si>
+  <si>
+    <t>0012968363</t>
+  </si>
+  <si>
+    <t>0012765489</t>
+  </si>
+  <si>
+    <t>0012765488</t>
+  </si>
+  <si>
+    <t>0012968362</t>
+  </si>
+  <si>
+    <t>0012765492</t>
+  </si>
+  <si>
+    <t>0012968360</t>
+  </si>
+  <si>
+    <t>0012765491</t>
+  </si>
+  <si>
+    <t>0012968364</t>
+  </si>
+  <si>
+    <t>0012765493</t>
+  </si>
+  <si>
+    <t>0012968359</t>
+  </si>
+  <si>
+    <t>принтер</t>
+  </si>
+  <si>
     <t>1.1</t>
   </si>
   <si>
-    <t>0012765490</t>
-  </si>
-  <si>
-    <t>0012968363</t>
-  </si>
-  <si>
     <t>1.2</t>
   </si>
   <si>
-    <t>0012765489</t>
-  </si>
-  <si>
     <t>1.3</t>
   </si>
   <si>
-    <t>0012765488</t>
-  </si>
-  <si>
-    <t>0012968362</t>
-  </si>
-  <si>
     <t>1.4</t>
   </si>
   <si>
-    <t>0012765492</t>
-  </si>
-  <si>
-    <t>0012968360</t>
-  </si>
-  <si>
     <t>1.5</t>
   </si>
   <si>
-    <t>0012765491</t>
-  </si>
-  <si>
-    <t>0012968364</t>
-  </si>
-  <si>
     <t>1.6</t>
-  </si>
-  <si>
-    <t>0012765493</t>
-  </si>
-  <si>
-    <t>0012968359</t>
-  </si>
-  <si>
-    <t>принтер</t>
   </si>
 </sst>
 </file>
@@ -118,12 +118,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -420,71 +423,71 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>